<commit_message>
Replace estimated loss with verified ad balance
</commit_message>
<xml_diff>
--- a/2026_09-2027_03_광고예산_ROI_흑자전환계획.xlsx
+++ b/2026_09-2027_03_광고예산_ROI_흑자전환계획.xlsx
@@ -219,55 +219,57 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>기준일</t>
+          <t>확정 집계 기간</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2025-11~2026-08-17</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>현재 Total Revenue</t>
+          <t>누적 Total Revenue</t>
         </is>
       </c>
       <c r="D3" s="4">
-        <v>25439.99</v>
+        <v>72904.18</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>현재 광고비</t>
+          <t>누적 광고비</t>
         </is>
       </c>
       <c r="F3" s="4">
-        <v>35235.56</v>
+        <v>135103.52</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>현재 관리 ROI</t>
-        </is>
-      </c>
-      <c r="B4" s="5">
-        <v>0.72</v>
+          <t>정확한 누적 광고수지</t>
+        </is>
+      </c>
+      <c r="B4" s="11">
+        <v>-62199.34</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>마감 누적 적자(7월)</t>
-        </is>
-      </c>
-      <c r="D4" s="4">
-        <v>-66111.69</v>
+          <t>정확한 누적 ROI</t>
+        </is>
+      </c>
+      <c r="D4" s="5">
+        <v>0.5396171765176807</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>8월 포함 보수적 누적</t>
-        </is>
-      </c>
-      <c r="F4" s="4">
-        <v>-89794.06</v>
+          <t>회계상 누적 순손실</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>원가원장 필요</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
@@ -305,7 +307,7 @@
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>월 흑자 목표</t>
+          <t>월 추정흑자 목표</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -315,12 +317,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>누적 흑자 목표</t>
+          <t>누적 광고수지 회복</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>2027년 2월</t>
+          <t>2026년 12월</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -547,8 +549,9 @@
     <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -607,15 +610,20 @@
           <t/>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>시작 누적손익</t>
+          <t>시작 누적 광고수지</t>
         </is>
       </c>
       <c r="B2" s="11">
-        <v>-89794.06</v>
+        <v>-62199.34</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -635,14 +643,14 @@
           <t>Total Revenue ÷ 광고비</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>회계 누적손익</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>원가원장 입력 전 확정 불가</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -656,6 +664,11 @@
         </is>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -704,15 +717,20 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>예상 누적손익</t>
+          <t>월 광고수지</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>누적 광고수지</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>집행 조건</t>
         </is>
@@ -750,15 +768,19 @@
         <v>-741.779799182983</v>
       </c>
       <c r="I5" s="4">
-        <f>$B$2+H5</f>
-        <v>-90535.83979918298</v>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
+        <f>F5-B5</f>
+        <v>6400.0</v>
+      </c>
+      <c r="J5" s="4">
+        <f>$B$2+I5</f>
+        <v>-55799.34</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>전환 단계</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>ROI 1.2 이상일 때 예비액 집행</t>
         </is>
@@ -796,15 +818,19 @@
         <v>6630.726797832442</v>
       </c>
       <c r="I6" s="4">
-        <f>I5+H6</f>
-        <v>-83905.11300135055</v>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>월 흑자</t>
-        </is>
+        <f>F6-B6</f>
+        <v>15000.0</v>
+      </c>
+      <c r="J6" s="4">
+        <f>J5+I6</f>
+        <v>-40799.34</v>
       </c>
       <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>월 추정흑자</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>9월 목표 달성 광고 중심 재배분</t>
         </is>
@@ -842,15 +868,19 @@
         <v>13026.414013572334</v>
       </c>
       <c r="I7" s="4">
-        <f>I6+H7</f>
-        <v>-70878.69898777822</v>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>월 흑자</t>
-        </is>
+        <f>F7-B7</f>
+        <v>22400.0</v>
+      </c>
+      <c r="J7" s="4">
+        <f>J6+I7</f>
+        <v>-18399.339999999997</v>
       </c>
       <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>월 추정흑자</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>상품별 기여이익 플러스 광고만 증액</t>
         </is>
@@ -888,15 +918,19 @@
         <v>18445.281848036695</v>
       </c>
       <c r="I8" s="4">
-        <f>I7+H8</f>
-        <v>-52433.41713974152</v>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>월 흑자</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
+        <f>F8-B8</f>
+        <v>28600.0</v>
+      </c>
+      <c r="J8" s="8">
+        <f>J7+I8</f>
+        <v>10200.660000000003</v>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>광고수지 회복</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>ROI 2.0 미만 광고 즉시 감액</t>
         </is>
@@ -934,15 +968,19 @@
         <v>24840.96906377659</v>
       </c>
       <c r="I9" s="4">
-        <f>I8+H9</f>
-        <v>-27592.44807596493</v>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>월 흑자</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
+        <f>F9-B9</f>
+        <v>36000.0</v>
+      </c>
+      <c r="J9" s="8">
+        <f>J8+I9</f>
+        <v>46200.66</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>광고수지 회복</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>주간 ROI 2.5 이상 유지</t>
         </is>
@@ -979,18 +1017,22 @@
         <f>F10-B10-G10</f>
         <v>28143.39490547729</v>
       </c>
-      <c r="I10" s="8">
-        <f>I9+H10</f>
-        <v>550.9468295123588</v>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>누적 흑자</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>누적 흑자 전환 확인</t>
+      <c r="I10" s="4">
+        <f>F10-B10</f>
+        <v>39599.99999999999</v>
+      </c>
+      <c r="J10" s="8">
+        <f>J9+I10</f>
+        <v>85800.66</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>광고수지 회복</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>월 마감 원가 입력 후 회계 손익 확인</t>
         </is>
       </c>
     </row>
@@ -1025,27 +1067,31 @@
         <f>F11-B11-G11</f>
         <v>31725.065970154246</v>
       </c>
-      <c r="I11" s="8">
-        <f>I10+H11</f>
-        <v>32276.012799666605</v>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>누적 흑자</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="I11" s="4">
+        <f>F11-B11</f>
+        <v>44000.0</v>
+      </c>
+      <c r="J11" s="8">
+        <f>J10+I11</f>
+        <v>129800.66</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>광고수지 회복</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>대표 목표 ROI 3.0 정착</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K11"/>
+  <autoFilter ref="A4:L11"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:I11">
+  <conditionalFormatting sqref="H5:J11">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -1262,7 +1308,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="68" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t/>
@@ -1270,7 +1316,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>9월 광고비는 최대 $32,000으로 승인받되 $24,000만 우선 집행합니다. 목표 ROI와 상품별 기여이익을 충족할 때만 예비액 $8,000을 단계적으로 사용합니다. 2027년 2월 누적 흑자, 3월 ROI 3.0을 목표로 관리합니다.</t>
+          <t>9월 광고비는 최대 $32,000으로 승인받되 $24,000만 우선 집행합니다. 목표 ROI와 상품별 기여이익을 충족할 때만 예비액 $8,000을 단계적으로 사용합니다. 누적 광고수지는 2026년 12월 회복, ROI 3.0은 2027년 3월을 목표로 합니다. 회계상 누적 순손실은 원가원장 입력 후 확정합니다.</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1301,7 +1347,7 @@
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="41" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1395,130 +1441,174 @@
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>7월까지 누적</t>
+          <t>누적 Total Revenue</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>assets/monthly-data.js 및 월별 Finance 원본</t>
+          <t>월별 Finance 원본 + 8월 income 원본</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>2025-11~2026-07</t>
+          <t>2025-11~2026-08-17</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>추정 누적손익 -$66,111.69</t>
+          <t>$72,904.18</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>비광고비율</t>
+          <t>누적 광고비</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Admin 비용 스냅샷</t>
+          <t>월별 Campaign 원본 + ads.tiktok.csv</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>현재 계획 가정</t>
+          <t>2025-11~2026-08-17</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>$13,559 ÷ $72,904.18 = 18.598%</t>
+          <t>$135,103.52</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>8월 포함 누적</t>
+          <t>정확한 누적 광고수지</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>정산액과 8/17까지 광고비 결합</t>
+          <t>Total Revenue - 광고비</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>컷오프 정렬</t>
+          <t>2025-11~2026-08-17</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>보수적 누적 -$89,794.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+          <t>-$62,199.34 · 누적 ROI 0.54x</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>비광고비율</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Admin 비용 스냅샷</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>현재 계획 가정</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>$13,559 ÷ $72,904.18 = 18.598%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>확인된 정산현금</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>월별 Finance Reports</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>2025-11~2026-06</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>$19,620.79 정산액 - $65,852.86 광고비 = -$46,232.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>검증 제한</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>8월 매출과 광고비의 종료일이 하루 다릅니다. 누적 손익은 의사결정용 보수적 추정이며 월 마감 확정치가 아닙니다.</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>제품 원가·시딩·수수료·물류비의 실제 월 마감 원장이 연결되면 비광고비 추정치를 실제값으로 교체해야 합니다.</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>누적 광고수지 -$62,199.34는 Total Revenue와 광고비 원본을 동일 종료일로 맞춘 정확한 값입니다. 회계상 순손실과는 다릅니다.</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>회계상 누적 순손실을 확정하려면 7월 정산액 원본과 월별 실제 제품 원가·외부 시딩·물류·기타 운영비 원장이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1527,9 +1617,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>

</xml_diff>